<commit_message>
Replace public workbook with verified final 11-sheet edition
</commit_message>
<xml_diff>
--- a/data/Hew_Underwriting_Public_Edition_2026.xlsx
+++ b/data/Hew_Underwriting_Public_Edition_2026.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdf84469414c449a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R92e9f91260594ac0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lease Economics" sheetId="3" r:id="Re69e95b471244c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pro Forma" sheetId="4" r:id="R4b9f9e1a00274962"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="5" r:id="R4626367bf8ab41b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Evidence" sheetId="6" r:id="Rba0b4bf2d4e5465f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hew Tax Evidence" sheetId="7" r:id="R29cd87ee6540449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand" sheetId="8" r:id="Ra2cbecc40cd94669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="R459a2efe88704fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="10" r:id="Rb52cc76139a5413e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R25beeab736f84aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R2d2069bbeac34f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lease Economics" sheetId="3" r:id="R4beb734ce8fa451c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pro Forma" sheetId="4" r:id="R63e684a73e79400e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="5" r:id="R6b8fab016b5242db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Evidence" sheetId="6" r:id="R5e622f43e8c0414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hew Tax Evidence" sheetId="7" r:id="R067cd14aafb34334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand" sheetId="8" r:id="Rc5cffe83c87742d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="R4be26eb0d3164d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="10" r:id="Rdd812a3024b64dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affordable Housing" sheetId="11" r:id="R5b50989d0e314999"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="12">
+  <x:numFmts count="17">
     <x:numFmt numFmtId="200" formatCode="#,##0;(#,##0);–"/>
     <x:numFmt numFmtId="201" formatCode="  @"/>
     <x:numFmt numFmtId="202" formatCode="0.0%;(0.0%);–"/>
@@ -35,8 +36,13 @@
     <x:numFmt numFmtId="209" formatCode="@"/>
     <x:numFmt numFmtId="210" formatCode="0.00;(0.00);–"/>
     <x:numFmt numFmtId="211" formatCode="0"/>
+    <x:numFmt numFmtId="212" formatCode="#,##0.0"/>
+    <x:numFmt numFmtId="213" formatCode="#,##0"/>
+    <x:numFmt numFmtId="214" formatCode="0.0%"/>
+    <x:numFmt numFmtId="215" formatCode="$#,##0;($#,##0)"/>
+    <x:numFmt numFmtId="216" formatCode="#,##0.00;(#,##0.00);–"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -75,8 +81,71 @@
       <x:color rgb="FF1556A7"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF263D5A"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF67788A"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1E3554"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2563A6"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF2563A6"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF156B54"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3554"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF67788A"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +167,36 @@
         <x:fgColor rgb="FFFFF4D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3554"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EFF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F3EE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEBF5F0"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -111,7 +210,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -152,6 +251,50 @@
     <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="211" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="212" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="216" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -467,17 +610,17 @@
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="1" t="str">
-        <x:v>Building-wide broker channel share</x:v>
+        <x:v>Broker-sourced leases for the whole building</x:v>
       </x:c>
       <x:c r="B9" s="38" t="str">
-        <x:v>Unavailable</x:v>
+        <x:v>n.a.</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
-        <x:v>Unavailable Information</x:v>
+        <x:v>Not publicly available</x:v>
       </x:c>
       <x:c r="D9" s="3"/>
       <x:c r="E9" s="1" t="str">
-        <x:v>A complete leasing ledger is required.</x:v>
+        <x:v>Neither full-building new lease count nor broker channel share is verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
@@ -492,7 +635,7 @@
       </x:c>
       <x:c r="D10" s="3"/>
       <x:c r="E10" s="1" t="str">
-        <x:v>Listing counts cannot establish these building-wide rates.</x:v>
+        <x:v>Neither denominator can be recovered from listing counts or one brokerage data</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
@@ -584,7 +727,7 @@
       </x:c>
       <x:c r="C18" s="3" t="n">
         <x:f>'Lease Economics'!C8</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D18" s="3"/>
       <x:c r="E18" s="1" t="str">
@@ -610,7 +753,7 @@
       </x:c>
       <x:c r="C20" s="20" t="n">
         <x:f>'Lease Economics'!C20</x:f>
-        <x:v>5446200.375</x:v>
+        <x:v>5395744.271875</x:v>
       </x:c>
       <x:c r="D20" s="3"/>
       <x:c r="E20" s="1" t="str">
@@ -627,7 +770,7 @@
       </x:c>
       <x:c r="C21" s="20" t="n">
         <x:f>'Lease Economics'!C21+'Lease Economics'!C22</x:f>
-        <x:v>-1123386.01125</x:v>
+        <x:v>-1121872.32815625</x:v>
       </x:c>
       <x:c r="D21" s="3"/>
       <x:c r="E21" s="1" t="str">
@@ -644,7 +787,7 @@
       </x:c>
       <x:c r="C22" s="20" t="n">
         <x:f>'Lease Economics'!C25</x:f>
-        <x:v>-839051.0056971824</x:v>
+        <x:v>-829551.3641921398</x:v>
       </x:c>
       <x:c r="D22" s="3"/>
       <x:c r="E22" s="1" t="str">
@@ -661,7 +804,7 @@
       </x:c>
       <x:c r="C23" s="26" t="n">
         <x:f>'Lease Economics'!C26</x:f>
-        <x:v>3483763.358052817</x:v>
+        <x:v>3444320.57952661</x:v>
       </x:c>
       <x:c r="D23" s="10"/>
       <x:c r="E23" s="9" t="str">
@@ -678,7 +821,7 @@
       </x:c>
       <x:c r="C24" s="20" t="n">
         <x:f>'Lease Economics'!C30</x:f>
-        <x:v>3339369.608052817</x:v>
+        <x:v>3300755.11077661</x:v>
       </x:c>
       <x:c r="D24" s="3"/>
       <x:c r="E24" s="1" t="str">
@@ -721,7 +864,7 @@
       </x:c>
       <x:c r="C27" s="26" t="n">
         <x:f>'Pro Forma'!C35</x:f>
-        <x:v>66995449.19332341</x:v>
+        <x:v>66236934.22166558</x:v>
       </x:c>
       <x:c r="D27" s="10"/>
       <x:c r="E27" s="9" t="str">
@@ -738,7 +881,7 @@
       </x:c>
       <x:c r="C28" s="26" t="n">
         <x:f>'Pro Forma'!C39</x:f>
-        <x:v>12286903.747853063</x:v>
+        <x:v>13045418.71951089</x:v>
       </x:c>
       <x:c r="D28" s="10"/>
       <x:c r="E28" s="9" t="str">
@@ -755,7 +898,7 @@
       </x:c>
       <x:c r="C29" s="27" t="n">
         <x:f>'Pro Forma'!C36</x:f>
-        <x:v>0.04394122057196757</x:v>
+        <x:v>0.043443722994474236</x:v>
       </x:c>
       <x:c r="D29" s="3"/>
       <x:c r="E29" s="1" t="str">
@@ -851,7 +994,7 @@
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
       <x:c r="A39" s="1" t="str">
-        <x:v>Report observations with their date and source; do not infer building-wide activity from partial records.</x:v>
+        <x:v>Report observations with their year and source; avoid publicly identifying brokerage production without consent.</x:v>
       </x:c>
       <x:c r="B39" s="3"/>
       <x:c r="C39" s="3"/>
@@ -886,7 +1029,7 @@
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Hew Public-Data Research — Final Workbook Guide (26 October 2026)</x:v>
+        <x:v>Hew Public-Data Research — Public Edition, Revised 27 October 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
@@ -941,12 +1084,12 @@
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" t="str">
-        <x:v>Broker commissions apply only to broker-sourced new tenants; the complete channel mix is unavailable.</x:v>
+        <x:v>Broker commissions are modeled for broker-sourced new tenants only. Full-building broker penetration is unknown.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" t="str">
-        <x:v>Public edition: confidential transaction records are excluded. Financial model assumptions and calculations are retained.</x:v>
+        <x:v>No private brokerage production, executed Hew rent roll or firm-specific transaction information is included.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
@@ -996,7 +1139,7 @@
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" t="str">
-        <x:v>The 17% restricted + 3% voucher set-aside is one example of city policy; hypothetical rent and voucher payments need compliance review.</x:v>
+        <x:v>The hypothetical 150-home mixed-income option now uses a transparent 26 restricted / 5 voucher ROUND-UP scenario; see Affordable Housing.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
@@ -1026,16 +1169,1486 @@
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" t="str">
-        <x:v>Summary → Inputs → Lease Economics → Pro Forma → Sensitivity → Market Evidence → Hew Tax Evidence → Demand → Audit.</x:v>
+        <x:v>Summary → Inputs → Lease Economics → Pro Forma → Sensitivity → Affordable Housing → Market Evidence → Hew Tax Evidence → Demand → Audit.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" t="str">
-        <x:v>The earlier 2026 Excel was updated using newly verified FY2026 Boston parcel taxes; earlier versions remain in file history.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="25" customHeight="1"/>
+        <x:v>Change Affordable Housing B21 to switch voucher rent benchmarks. All public outputs are hypothetical, not Hew actual NOI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="25" customHeight="1">
+      <x:c r="A31" t="str">
+        <x:v>Restricted rent uses published 2025 City IDP 60% AMI standard-size limits and an ASSUMED unit mix; 2026 IDP limits not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>BHA gross payment standards are not project contract rent; verify tenant-paid utilities and BHA rent-reasonableness assessment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>All mixed-income totals update through formulas, including NOI, property tax estimate, value, yield and gap.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>Illustrative 48 Studio / 67 one-bedroom / 35 two-bedroom mix extrapolated from a user-recorded 123-listing sample, NOT the building rent roll.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>The $3,875 market rent is a single blended input across market-rate unit types; restricted/voucher rent varies by bedroom.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="42" t="str">
+        <x:v>Affordable Housing | Bedroom and Voucher Revenue Schedule</x:v>
+      </x:c>
+      <x:c r="B1" s="42"/>
+      <x:c r="C1" s="42"/>
+      <x:c r="D1" s="42"/>
+      <x:c r="E1" s="42"/>
+      <x:c r="F1" s="42"/>
+      <x:c r="G1" s="42"/>
+      <x:c r="H1" s="42"/>
+      <x:c r="I1" s="42"/>
+      <x:c r="J1" s="42"/>
+      <x:c r="K1" s="42"/>
+      <x:c r="L1" s="42"/>
+      <x:c r="M1" s="42"/>
+      <x:c r="N1" s="42"/>
+      <x:c r="O1" s="42"/>
+      <x:c r="P1" s="42"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="44" t="str">
+        <x:v>Separate illustrative 150-home Brighton development, NOT Hew actual restricted inventory or contract rents.</x:v>
+      </x:c>
+      <x:c r="B2" s="44"/>
+      <x:c r="C2" s="44"/>
+      <x:c r="D2" s="44"/>
+      <x:c r="E2" s="44"/>
+      <x:c r="F2" s="44"/>
+      <x:c r="G2" s="44"/>
+      <x:c r="H2" s="44"/>
+      <x:c r="I2" s="44"/>
+      <x:c r="J2" s="44"/>
+      <x:c r="K2" s="44"/>
+      <x:c r="L2" s="44"/>
+      <x:c r="M2" s="44"/>
+      <x:c r="N2" s="44"/>
+      <x:c r="O2" s="44"/>
+      <x:c r="P2" s="44"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="40"/>
+      <x:c r="B3" s="40"/>
+      <x:c r="C3" s="40"/>
+      <x:c r="D3" s="40"/>
+      <x:c r="E3" s="40"/>
+      <x:c r="F3" s="40"/>
+      <x:c r="G3" s="40"/>
+      <x:c r="H3" s="40"/>
+      <x:c r="I3" s="40"/>
+      <x:c r="J3" s="40"/>
+      <x:c r="K3" s="40"/>
+      <x:c r="L3" s="40"/>
+      <x:c r="M3" s="40"/>
+      <x:c r="N3" s="40"/>
+      <x:c r="O3" s="40"/>
+      <x:c r="P3" s="40"/>
+    </x:row>
+    <x:row r="4" ht="25" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>POLICY ROUNDING | MODEL OPTION</x:v>
+      </x:c>
+      <x:c r="B4" s="45"/>
+      <x:c r="C4" s="45"/>
+      <x:c r="D4" s="45"/>
+      <x:c r="E4" s="45"/>
+      <x:c r="F4" s="45"/>
+      <x:c r="G4" s="45"/>
+      <x:c r="H4" s="45"/>
+      <x:c r="I4" s="45"/>
+      <x:c r="J4" s="45"/>
+      <x:c r="K4" s="45"/>
+      <x:c r="L4" s="45"/>
+      <x:c r="M4" s="45"/>
+      <x:c r="N4" s="45"/>
+      <x:c r="O4" s="45"/>
+      <x:c r="P4" s="45"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="47" t="str">
+        <x:v>Driver</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Evidence class</x:v>
+      </x:c>
+      <x:c r="E5" s="40"/>
+      <x:c r="F5" s="40"/>
+      <x:c r="G5" s="40"/>
+      <x:c r="H5" s="40"/>
+      <x:c r="I5" s="40"/>
+      <x:c r="J5" s="40"/>
+      <x:c r="K5" s="40"/>
+      <x:c r="L5" s="40"/>
+      <x:c r="M5" s="40"/>
+      <x:c r="N5" s="40"/>
+      <x:c r="O5" s="40"/>
+      <x:c r="P5" s="40"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="40" t="str">
+        <x:v>Project homes</x:v>
+      </x:c>
+      <x:c r="B6" s="48" t="n">
+        <x:f>Inputs!$B$6</x:f>
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>Illustrative site scale</x:v>
+      </x:c>
+      <x:c r="D6" s="40" t="str">
+        <x:v>Model input</x:v>
+      </x:c>
+      <x:c r="E6" s="40"/>
+      <x:c r="F6" s="40"/>
+      <x:c r="G6" s="40"/>
+      <x:c r="H6" s="40"/>
+      <x:c r="I6" s="40"/>
+      <x:c r="J6" s="40"/>
+      <x:c r="K6" s="40"/>
+      <x:c r="L6" s="40"/>
+      <x:c r="M6" s="40"/>
+      <x:c r="N6" s="40"/>
+      <x:c r="O6" s="40"/>
+      <x:c r="P6" s="40"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="40" t="str">
+        <x:v>Restricted share</x:v>
+      </x:c>
+      <x:c r="B7" s="50" t="n">
+        <x:f>Inputs!$B$18</x:f>
+        <x:v>0.17</x:v>
+      </x:c>
+      <x:c r="C7" s="40" t="str">
+        <x:v>Option B 17%</x:v>
+      </x:c>
+      <x:c r="D7" s="40" t="str">
+        <x:v>Policy scenario</x:v>
+      </x:c>
+      <x:c r="E7" s="40"/>
+      <x:c r="F7" s="40"/>
+      <x:c r="G7" s="40"/>
+      <x:c r="H7" s="40"/>
+      <x:c r="I7" s="40"/>
+      <x:c r="J7" s="40"/>
+      <x:c r="K7" s="40"/>
+      <x:c r="L7" s="40"/>
+      <x:c r="M7" s="40"/>
+      <x:c r="N7" s="40"/>
+      <x:c r="O7" s="40"/>
+      <x:c r="P7" s="40"/>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="40" t="str">
+        <x:v>Voucher share</x:v>
+      </x:c>
+      <x:c r="B8" s="50" t="n">
+        <x:f>Inputs!$B$19</x:f>
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="C8" s="40" t="str">
+        <x:v>Additional 3%</x:v>
+      </x:c>
+      <x:c r="D8" s="40" t="str">
+        <x:v>Policy scenario</x:v>
+      </x:c>
+      <x:c r="E8" s="40"/>
+      <x:c r="F8" s="40"/>
+      <x:c r="G8" s="40"/>
+      <x:c r="H8" s="40"/>
+      <x:c r="I8" s="40"/>
+      <x:c r="J8" s="40"/>
+      <x:c r="K8" s="40"/>
+      <x:c r="L8" s="40"/>
+      <x:c r="M8" s="40"/>
+      <x:c r="N8" s="40"/>
+      <x:c r="O8" s="40"/>
+      <x:c r="P8" s="40"/>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="40" t="str">
+        <x:v>Theoretical restricted homes</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="n">
+        <x:f>B6*B7</x:f>
+        <x:v>25.500000000000004</x:v>
+      </x:c>
+      <x:c r="C9" s="40" t="str">
+        <x:v>25.5 at 150 homes</x:v>
+      </x:c>
+      <x:c r="D9" s="40" t="str">
+        <x:v>Derived</x:v>
+      </x:c>
+      <x:c r="E9" s="40"/>
+      <x:c r="F9" s="40"/>
+      <x:c r="G9" s="40"/>
+      <x:c r="H9" s="40"/>
+      <x:c r="I9" s="40"/>
+      <x:c r="J9" s="40"/>
+      <x:c r="K9" s="40"/>
+      <x:c r="L9" s="40"/>
+      <x:c r="M9" s="40"/>
+      <x:c r="N9" s="40"/>
+      <x:c r="O9" s="40"/>
+      <x:c r="P9" s="40"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="40" t="str">
+        <x:v>Theoretical voucher homes</x:v>
+      </x:c>
+      <x:c r="B10" s="48" t="n">
+        <x:f>B6*B8</x:f>
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>4.5 at 150 homes</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="str">
+        <x:v>Derived</x:v>
+      </x:c>
+      <x:c r="E10" s="40"/>
+      <x:c r="F10" s="40"/>
+      <x:c r="G10" s="40"/>
+      <x:c r="H10" s="40"/>
+      <x:c r="I10" s="40"/>
+      <x:c r="J10" s="40"/>
+      <x:c r="K10" s="40"/>
+      <x:c r="L10" s="40"/>
+      <x:c r="M10" s="40"/>
+      <x:c r="N10" s="40"/>
+      <x:c r="O10" s="40"/>
+      <x:c r="P10" s="40"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="52" t="str">
+        <x:v>Restricted homes: rounded up</x:v>
+      </x:c>
+      <x:c r="B11" s="53" t="n">
+        <x:f>ROUNDUP(B9,0)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C11" s="40" t="str">
+        <x:v>26 units</x:v>
+      </x:c>
+      <x:c r="D11" s="40" t="str">
+        <x:v>Illustrative rounding</x:v>
+      </x:c>
+      <x:c r="E11" s="40"/>
+      <x:c r="F11" s="40"/>
+      <x:c r="G11" s="40"/>
+      <x:c r="H11" s="40"/>
+      <x:c r="I11" s="40"/>
+      <x:c r="J11" s="40"/>
+      <x:c r="K11" s="40"/>
+      <x:c r="L11" s="40"/>
+      <x:c r="M11" s="40"/>
+      <x:c r="N11" s="40"/>
+      <x:c r="O11" s="40"/>
+      <x:c r="P11" s="40"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="52" t="str">
+        <x:v>Voucher homes: rounded up</x:v>
+      </x:c>
+      <x:c r="B12" s="53" t="n">
+        <x:f>ROUNDUP(B10,0)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C12" s="40" t="str">
+        <x:v>5 units</x:v>
+      </x:c>
+      <x:c r="D12" s="40" t="str">
+        <x:v>Illustrative rounding</x:v>
+      </x:c>
+      <x:c r="E12" s="40"/>
+      <x:c r="F12" s="40"/>
+      <x:c r="G12" s="40"/>
+      <x:c r="H12" s="40"/>
+      <x:c r="I12" s="40"/>
+      <x:c r="J12" s="40"/>
+      <x:c r="K12" s="40"/>
+      <x:c r="L12" s="40"/>
+      <x:c r="M12" s="40"/>
+      <x:c r="N12" s="40"/>
+      <x:c r="O12" s="40"/>
+      <x:c r="P12" s="40"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="52" t="str">
+        <x:v>Total designated homes</x:v>
+      </x:c>
+      <x:c r="B13" s="53" t="n">
+        <x:f>SUM(B11:B12)</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C13" s="40" t="str">
+        <x:v>No double-counting</x:v>
+      </x:c>
+      <x:c r="D13" s="40" t="str">
+        <x:v>Derived</x:v>
+      </x:c>
+      <x:c r="E13" s="40"/>
+      <x:c r="F13" s="40"/>
+      <x:c r="G13" s="40"/>
+      <x:c r="H13" s="40"/>
+      <x:c r="I13" s="40"/>
+      <x:c r="J13" s="40"/>
+      <x:c r="K13" s="40"/>
+      <x:c r="L13" s="40"/>
+      <x:c r="M13" s="40"/>
+      <x:c r="N13" s="40"/>
+      <x:c r="O13" s="40"/>
+      <x:c r="P13" s="40"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="52" t="str">
+        <x:v>Residual market homes</x:v>
+      </x:c>
+      <x:c r="B14" s="53" t="n">
+        <x:f>B6-B13</x:f>
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>Project total less set-asides</x:v>
+      </x:c>
+      <x:c r="D14" s="40" t="str">
+        <x:v>Derived</x:v>
+      </x:c>
+      <x:c r="E14" s="40"/>
+      <x:c r="F14" s="40"/>
+      <x:c r="G14" s="40"/>
+      <x:c r="H14" s="40"/>
+      <x:c r="I14" s="40"/>
+      <x:c r="J14" s="40"/>
+      <x:c r="K14" s="40"/>
+      <x:c r="L14" s="40"/>
+      <x:c r="M14" s="40"/>
+      <x:c r="N14" s="40"/>
+      <x:c r="O14" s="40"/>
+      <x:c r="P14" s="40"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="52" t="str">
+        <x:v>Effective combined set-aside</x:v>
+      </x:c>
+      <x:c r="B15" s="54" t="n">
+        <x:f>B13/B6</x:f>
+        <x:v>0.20666666666666667</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>31 / 150 = 20.67%</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>Derived</x:v>
+      </x:c>
+      <x:c r="E15" s="40"/>
+      <x:c r="F15" s="40"/>
+      <x:c r="G15" s="40"/>
+      <x:c r="H15" s="40"/>
+      <x:c r="I15" s="40"/>
+      <x:c r="J15" s="40"/>
+      <x:c r="K15" s="40"/>
+      <x:c r="L15" s="40"/>
+      <x:c r="M15" s="40"/>
+      <x:c r="N15" s="40"/>
+      <x:c r="O15" s="40"/>
+      <x:c r="P15" s="40"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="40" t="str">
+        <x:v>Round-up is one screening method; fraction-of-unit, floor area, fee options and applicability need counsel / City confirmation.</x:v>
+      </x:c>
+      <x:c r="B16" s="40"/>
+      <x:c r="C16" s="40"/>
+      <x:c r="D16" s="40"/>
+      <x:c r="E16" s="40"/>
+      <x:c r="F16" s="40"/>
+      <x:c r="G16" s="40"/>
+      <x:c r="H16" s="40"/>
+      <x:c r="I16" s="40"/>
+      <x:c r="J16" s="40"/>
+      <x:c r="K16" s="40"/>
+      <x:c r="L16" s="40"/>
+      <x:c r="M16" s="40"/>
+      <x:c r="N16" s="40"/>
+      <x:c r="O16" s="40"/>
+      <x:c r="P16" s="40"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="40" t="str">
+        <x:v>Hew (opened 2024) is NOT assumed to be subject to this hypothetical post-October-2024 project scenario.</x:v>
+      </x:c>
+      <x:c r="B17" s="40"/>
+      <x:c r="C17" s="40"/>
+      <x:c r="D17" s="40"/>
+      <x:c r="E17" s="40"/>
+      <x:c r="F17" s="40"/>
+      <x:c r="G17" s="40"/>
+      <x:c r="H17" s="40"/>
+      <x:c r="I17" s="40"/>
+      <x:c r="J17" s="40"/>
+      <x:c r="K17" s="40"/>
+      <x:c r="L17" s="40"/>
+      <x:c r="M17" s="40"/>
+      <x:c r="N17" s="40"/>
+      <x:c r="O17" s="40"/>
+      <x:c r="P17" s="40"/>
+    </x:row>
+    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="A18" s="45" t="str">
+        <x:v>REVENUE SENSITIVITY | EDITABLE DRIVERS</x:v>
+      </x:c>
+      <x:c r="B18" s="45"/>
+      <x:c r="C18" s="45"/>
+      <x:c r="D18" s="45"/>
+      <x:c r="E18" s="45"/>
+      <x:c r="F18" s="45"/>
+      <x:c r="G18" s="45"/>
+      <x:c r="H18" s="45"/>
+      <x:c r="I18" s="45"/>
+      <x:c r="J18" s="45"/>
+      <x:c r="K18" s="45"/>
+      <x:c r="L18" s="45"/>
+      <x:c r="M18" s="45"/>
+      <x:c r="N18" s="45"/>
+      <x:c r="O18" s="45"/>
+      <x:c r="P18" s="45"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="40" t="str">
+        <x:v>AMI treatment</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>60% AMI assumed</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>Uniform AMI is not legally validated.</x:v>
+      </x:c>
+      <x:c r="D19" s="40"/>
+      <x:c r="E19" s="40"/>
+      <x:c r="F19" s="40"/>
+      <x:c r="G19" s="40"/>
+      <x:c r="H19" s="40"/>
+      <x:c r="I19" s="40"/>
+      <x:c r="J19" s="40"/>
+      <x:c r="K19" s="40"/>
+      <x:c r="L19" s="40"/>
+      <x:c r="M19" s="40"/>
+      <x:c r="N19" s="40"/>
+      <x:c r="O19" s="40"/>
+      <x:c r="P19" s="40"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="40" t="str">
+        <x:v>2025 IDP limits</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>2025 verified</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>Confirm 2026 project-specific ceilings.</x:v>
+      </x:c>
+      <x:c r="D20" s="40"/>
+      <x:c r="E20" s="40"/>
+      <x:c r="F20" s="40"/>
+      <x:c r="G20" s="40"/>
+      <x:c r="H20" s="40"/>
+      <x:c r="I20" s="40"/>
+      <x:c r="J20" s="40"/>
+      <x:c r="K20" s="40"/>
+      <x:c r="L20" s="40"/>
+      <x:c r="M20" s="40"/>
+      <x:c r="N20" s="40"/>
+      <x:c r="O20" s="40"/>
+      <x:c r="P20" s="40"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="40" t="str">
+        <x:v>Voucher income mode (1 / 2)</x:v>
+      </x:c>
+      <x:c r="B21" s="56" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>1 = market; 2 = BHA benchmark</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>Neither is approved contract rent.</x:v>
+      </x:c>
+      <x:c r="E21" s="40"/>
+      <x:c r="F21" s="40"/>
+      <x:c r="G21" s="40"/>
+      <x:c r="H21" s="40"/>
+      <x:c r="I21" s="40"/>
+      <x:c r="J21" s="40"/>
+      <x:c r="K21" s="40"/>
+      <x:c r="L21" s="40"/>
+      <x:c r="M21" s="40"/>
+      <x:c r="N21" s="40"/>
+      <x:c r="O21" s="40"/>
+      <x:c r="P21" s="40"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="40" t="str">
+        <x:v>Voucher utility allowance: Studio</x:v>
+      </x:c>
+      <x:c r="B22" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="40"/>
+      <x:c r="D22" s="40" t="str">
+        <x:v>Zero means unverified / not yet deducted; change only with applicable BHA and MOH rules.</x:v>
+      </x:c>
+      <x:c r="E22" s="40"/>
+      <x:c r="F22" s="40"/>
+      <x:c r="G22" s="40"/>
+      <x:c r="H22" s="40"/>
+      <x:c r="I22" s="40"/>
+      <x:c r="J22" s="40"/>
+      <x:c r="K22" s="40"/>
+      <x:c r="L22" s="40"/>
+      <x:c r="M22" s="40"/>
+      <x:c r="N22" s="40"/>
+      <x:c r="O22" s="40"/>
+      <x:c r="P22" s="40"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="40" t="str">
+        <x:v>Voucher utility allowance: 1BR</x:v>
+      </x:c>
+      <x:c r="B23" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C23" s="40"/>
+      <x:c r="D23" s="40"/>
+      <x:c r="E23" s="40"/>
+      <x:c r="F23" s="40"/>
+      <x:c r="G23" s="40"/>
+      <x:c r="H23" s="40"/>
+      <x:c r="I23" s="40"/>
+      <x:c r="J23" s="40"/>
+      <x:c r="K23" s="40"/>
+      <x:c r="L23" s="40"/>
+      <x:c r="M23" s="40"/>
+      <x:c r="N23" s="40"/>
+      <x:c r="O23" s="40"/>
+      <x:c r="P23" s="40"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="40" t="str">
+        <x:v>Voucher utility allowance: 2BR</x:v>
+      </x:c>
+      <x:c r="B24" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C24" s="40"/>
+      <x:c r="D24" s="40"/>
+      <x:c r="E24" s="40"/>
+      <x:c r="F24" s="40"/>
+      <x:c r="G24" s="40"/>
+      <x:c r="H24" s="40"/>
+      <x:c r="I24" s="40"/>
+      <x:c r="J24" s="40"/>
+      <x:c r="K24" s="40"/>
+      <x:c r="L24" s="40"/>
+      <x:c r="M24" s="40"/>
+      <x:c r="N24" s="40"/>
+      <x:c r="O24" s="40"/>
+      <x:c r="P24" s="40"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="40" t="str">
+        <x:v>IDP allowance adjustment: Studio</x:v>
+      </x:c>
+      <x:c r="B25" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C25" s="40"/>
+      <x:c r="D25" s="40" t="str">
+        <x:v>Rents before project-specific utilities / compact-unit adjustments.</x:v>
+      </x:c>
+      <x:c r="E25" s="40"/>
+      <x:c r="F25" s="40"/>
+      <x:c r="G25" s="40"/>
+      <x:c r="H25" s="40"/>
+      <x:c r="I25" s="40"/>
+      <x:c r="J25" s="40"/>
+      <x:c r="K25" s="40"/>
+      <x:c r="L25" s="40"/>
+      <x:c r="M25" s="40"/>
+      <x:c r="N25" s="40"/>
+      <x:c r="O25" s="40"/>
+      <x:c r="P25" s="40"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="40" t="str">
+        <x:v>IDP allowance adjustment: 1BR</x:v>
+      </x:c>
+      <x:c r="B26" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C26" s="40"/>
+      <x:c r="D26" s="40"/>
+      <x:c r="E26" s="40"/>
+      <x:c r="F26" s="40"/>
+      <x:c r="G26" s="40"/>
+      <x:c r="H26" s="40"/>
+      <x:c r="I26" s="40"/>
+      <x:c r="J26" s="40"/>
+      <x:c r="K26" s="40"/>
+      <x:c r="L26" s="40"/>
+      <x:c r="M26" s="40"/>
+      <x:c r="N26" s="40"/>
+      <x:c r="O26" s="40"/>
+      <x:c r="P26" s="40"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="40" t="str">
+        <x:v>IDP allowance adjustment: 2BR</x:v>
+      </x:c>
+      <x:c r="B27" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C27" s="40"/>
+      <x:c r="D27" s="40"/>
+      <x:c r="E27" s="40"/>
+      <x:c r="F27" s="40"/>
+      <x:c r="G27" s="40"/>
+      <x:c r="H27" s="40"/>
+      <x:c r="I27" s="40"/>
+      <x:c r="J27" s="40"/>
+      <x:c r="K27" s="40"/>
+      <x:c r="L27" s="40"/>
+      <x:c r="M27" s="40"/>
+      <x:c r="N27" s="40"/>
+      <x:c r="O27" s="40"/>
+      <x:c r="P27" s="40"/>
+    </x:row>
+    <x:row r="28" ht="25" customHeight="1">
+      <x:c r="A28" s="45" t="str">
+        <x:v>BEDROOM MIX | UNIT-WEIGHTED REVENUE</x:v>
+      </x:c>
+      <x:c r="B28" s="45"/>
+      <x:c r="C28" s="45"/>
+      <x:c r="D28" s="45"/>
+      <x:c r="E28" s="45"/>
+      <x:c r="F28" s="45"/>
+      <x:c r="G28" s="45"/>
+      <x:c r="H28" s="45"/>
+      <x:c r="I28" s="45"/>
+      <x:c r="J28" s="45"/>
+      <x:c r="K28" s="45"/>
+      <x:c r="L28" s="45"/>
+      <x:c r="M28" s="45"/>
+      <x:c r="N28" s="45"/>
+      <x:c r="O28" s="45"/>
+      <x:c r="P28" s="45"/>
+    </x:row>
+    <x:row r="29" ht="41" customHeight="1">
+      <x:c r="A29" s="58" t="str">
+        <x:v>Bedrooms</x:v>
+      </x:c>
+      <x:c r="B29" s="58" t="str">
+        <x:v>All homes</x:v>
+      </x:c>
+      <x:c r="C29" s="58" t="str">
+        <x:v>Restricted</x:v>
+      </x:c>
+      <x:c r="D29" s="58" t="str">
+        <x:v>Voucher</x:v>
+      </x:c>
+      <x:c r="E29" s="58" t="str">
+        <x:v>Market</x:v>
+      </x:c>
+      <x:c r="F29" s="58" t="str">
+        <x:v>IDP 2025 60%</x:v>
+      </x:c>
+      <x:c r="G29" s="58" t="str">
+        <x:v>IDP allowance</x:v>
+      </x:c>
+      <x:c r="H29" s="58" t="str">
+        <x:v>Restricted net/mo</x:v>
+      </x:c>
+      <x:c r="I29" s="58" t="str">
+        <x:v>Restricted/yr</x:v>
+      </x:c>
+      <x:c r="J29" s="58" t="str">
+        <x:v>BHA 2026 02135</x:v>
+      </x:c>
+      <x:c r="K29" s="58" t="str">
+        <x:v>Voucher utility</x:v>
+      </x:c>
+      <x:c r="L29" s="58" t="str">
+        <x:v>BHA proxy/mo</x:v>
+      </x:c>
+      <x:c r="M29" s="58" t="str">
+        <x:v>Market proxy/mo</x:v>
+      </x:c>
+      <x:c r="N29" s="58" t="str">
+        <x:v>Selected voucher/mo</x:v>
+      </x:c>
+      <x:c r="O29" s="58" t="str">
+        <x:v>Voucher/yr</x:v>
+      </x:c>
+      <x:c r="P29" s="58" t="str">
+        <x:v>Mix check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="40" t="str">
+        <x:v>150-home mix extrapolated from user-observed 123 listings (approx. 32% / 45% / 24%). NOT Hew's verified full inventory.</x:v>
+      </x:c>
+      <x:c r="B30" s="40"/>
+      <x:c r="C30" s="40"/>
+      <x:c r="D30" s="40"/>
+      <x:c r="E30" s="40"/>
+      <x:c r="F30" s="40"/>
+      <x:c r="G30" s="40"/>
+      <x:c r="H30" s="40"/>
+      <x:c r="I30" s="40"/>
+      <x:c r="J30" s="40"/>
+      <x:c r="K30" s="40"/>
+      <x:c r="L30" s="40"/>
+      <x:c r="M30" s="40"/>
+      <x:c r="N30" s="40"/>
+      <x:c r="O30" s="40"/>
+      <x:c r="P30" s="40"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="40" t="str">
+        <x:v>Studio</x:v>
+      </x:c>
+      <x:c r="B31" s="64" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C31" s="64" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D31" s="64" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E31" s="49" t="n">
+        <x:f>B31-C31-D31</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F31" s="62" t="n">
+        <x:v>1266</x:v>
+      </x:c>
+      <x:c r="G31" s="63" t="n">
+        <x:f>B25</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="63" t="n">
+        <x:f>MAX(0,F31-G31)</x:f>
+        <x:v>1266</x:v>
+      </x:c>
+      <x:c r="I31" s="63" t="n">
+        <x:f>C31*H31*12</x:f>
+        <x:v>121536</x:v>
+      </x:c>
+      <x:c r="J31" s="62" t="n">
+        <x:v>2627</x:v>
+      </x:c>
+      <x:c r="K31" s="63" t="n">
+        <x:f>B22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="63" t="n">
+        <x:f>MAX(0,J31-K31)</x:f>
+        <x:v>2627</x:v>
+      </x:c>
+      <x:c r="M31" s="63" t="n">
+        <x:f>Inputs!$B$14</x:f>
+        <x:v>3875</x:v>
+      </x:c>
+      <x:c r="N31" s="63" t="n">
+        <x:f>IF($B$21=1,M31,L31)</x:f>
+        <x:v>2627</x:v>
+      </x:c>
+      <x:c r="O31" s="63" t="n">
+        <x:f>D31*N31*12</x:f>
+        <x:v>63048</x:v>
+      </x:c>
+      <x:c r="P31" s="49" t="n">
+        <x:f>B31-SUM(C31:E31)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="40" t="str">
+        <x:v>1 bedroom</x:v>
+      </x:c>
+      <x:c r="B32" s="64" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C32" s="64" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D32" s="64" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E32" s="49" t="n">
+        <x:f>B32-C32-D32</x:f>
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="F32" s="62" t="n">
+        <x:v>1484</x:v>
+      </x:c>
+      <x:c r="G32" s="63" t="n">
+        <x:f>B26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" s="63" t="n">
+        <x:f>MAX(0,F32-G32)</x:f>
+        <x:v>1484</x:v>
+      </x:c>
+      <x:c r="I32" s="63" t="n">
+        <x:f>C32*H32*12</x:f>
+        <x:v>213696</x:v>
+      </x:c>
+      <x:c r="J32" s="62" t="n">
+        <x:v>2757</x:v>
+      </x:c>
+      <x:c r="K32" s="63" t="n">
+        <x:f>B23</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="63" t="n">
+        <x:f>MAX(0,J32-K32)</x:f>
+        <x:v>2757</x:v>
+      </x:c>
+      <x:c r="M32" s="63" t="n">
+        <x:f>Inputs!$B$14</x:f>
+        <x:v>3875</x:v>
+      </x:c>
+      <x:c r="N32" s="63" t="n">
+        <x:f>IF($B$21=1,M32,L32)</x:f>
+        <x:v>2757</x:v>
+      </x:c>
+      <x:c r="O32" s="63" t="n">
+        <x:f>D32*N32*12</x:f>
+        <x:v>66168</x:v>
+      </x:c>
+      <x:c r="P32" s="49" t="n">
+        <x:f>B32-SUM(C32:E32)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="40" t="str">
+        <x:v>2 bedrooms</x:v>
+      </x:c>
+      <x:c r="B33" s="64" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C33" s="64" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D33" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E33" s="49" t="n">
+        <x:f>B33-C33-D33</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F33" s="62" t="n">
+        <x:v>1680</x:v>
+      </x:c>
+      <x:c r="G33" s="63" t="n">
+        <x:f>B27</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H33" s="63" t="n">
+        <x:f>MAX(0,F33-G33)</x:f>
+        <x:v>1680</x:v>
+      </x:c>
+      <x:c r="I33" s="63" t="n">
+        <x:f>C33*H33*12</x:f>
+        <x:v>120960</x:v>
+      </x:c>
+      <x:c r="J33" s="62" t="n">
+        <x:v>3270</x:v>
+      </x:c>
+      <x:c r="K33" s="63" t="n">
+        <x:f>B24</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="63" t="n">
+        <x:f>MAX(0,J33-K33)</x:f>
+        <x:v>3270</x:v>
+      </x:c>
+      <x:c r="M33" s="63" t="n">
+        <x:f>Inputs!$B$14</x:f>
+        <x:v>3875</x:v>
+      </x:c>
+      <x:c r="N33" s="63" t="n">
+        <x:f>IF($B$21=1,M33,L33)</x:f>
+        <x:v>3270</x:v>
+      </x:c>
+      <x:c r="O33" s="63" t="n">
+        <x:f>D33*N33*12</x:f>
+        <x:v>39240</x:v>
+      </x:c>
+      <x:c r="P33" s="49" t="n">
+        <x:f>B33-SUM(C33:E33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="67" t="str">
+        <x:v>TOTAL / WEIGHTED</x:v>
+      </x:c>
+      <x:c r="B34" s="68" t="n">
+        <x:f>SUM(B31:B33)</x:f>
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C34" s="68" t="n">
+        <x:f>SUM(C31:C33)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D34" s="68" t="n">
+        <x:f>SUM(D31:D33)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E34" s="68" t="n">
+        <x:f>SUM(E31:E33)</x:f>
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F34" s="69"/>
+      <x:c r="G34" s="69"/>
+      <x:c r="H34" s="69" t="n">
+        <x:f>IF(C34&gt;0,I34/(C34*12),0)</x:f>
+        <x:v>1462.1538461538462</x:v>
+      </x:c>
+      <x:c r="I34" s="69" t="n">
+        <x:f>SUM(I31:I33)</x:f>
+        <x:v>456192</x:v>
+      </x:c>
+      <x:c r="J34" s="69"/>
+      <x:c r="K34" s="69"/>
+      <x:c r="L34" s="69" t="n">
+        <x:f>IF(D34&gt;0,SUMPRODUCT(D31:D33,L31:L33)/D34,0)</x:f>
+        <x:v>2807.6</x:v>
+      </x:c>
+      <x:c r="M34" s="69" t="n">
+        <x:f>Inputs!$B$14</x:f>
+        <x:v>3875</x:v>
+      </x:c>
+      <x:c r="N34" s="69" t="n">
+        <x:f>IF(D34&gt;0,O34/(D34*12),0)</x:f>
+        <x:v>2807.6</x:v>
+      </x:c>
+      <x:c r="O34" s="69" t="n">
+        <x:f>SUM(O31:O33)</x:f>
+        <x:v>168456</x:v>
+      </x:c>
+      <x:c r="P34" s="68" t="n">
+        <x:f>SUM(P31:P33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="40" t="str">
+        <x:v>2025 City IDP 60% AMI limits and 2026 BHA standards are independent references; no 2026 IDP rent sheet verified.</x:v>
+      </x:c>
+      <x:c r="B35" s="40"/>
+      <x:c r="C35" s="40"/>
+      <x:c r="D35" s="40"/>
+      <x:c r="E35" s="40"/>
+      <x:c r="F35" s="40"/>
+      <x:c r="G35" s="40"/>
+      <x:c r="H35" s="40"/>
+      <x:c r="I35" s="40"/>
+      <x:c r="J35" s="40"/>
+      <x:c r="K35" s="40"/>
+      <x:c r="L35" s="40"/>
+      <x:c r="M35" s="40"/>
+      <x:c r="N35" s="40"/>
+      <x:c r="O35" s="40"/>
+      <x:c r="P35" s="40"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="40" t="str">
+        <x:v>BHA payment standard is a gross-rent benchmark, NOT approved landlord rent. Utilities and rent reasonableness still apply.</x:v>
+      </x:c>
+      <x:c r="B36" s="40"/>
+      <x:c r="C36" s="40"/>
+      <x:c r="D36" s="40"/>
+      <x:c r="E36" s="40"/>
+      <x:c r="F36" s="40"/>
+      <x:c r="G36" s="40"/>
+      <x:c r="H36" s="40"/>
+      <x:c r="I36" s="40"/>
+      <x:c r="J36" s="40"/>
+      <x:c r="K36" s="40"/>
+      <x:c r="L36" s="40"/>
+      <x:c r="M36" s="40"/>
+      <x:c r="N36" s="40"/>
+      <x:c r="O36" s="40"/>
+      <x:c r="P36" s="40"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="40" t="str">
+        <x:v>Current mode:</x:v>
+      </x:c>
+      <x:c r="B37" s="40" t="str">
+        <x:f>IF(B21=1,"Market proxy (unverified)","BHA gross standard less assumed allowance (benchmark only)")</x:f>
+        <x:v>BHA gross standard less assumed allowance (benchmark only)</x:v>
+      </x:c>
+      <x:c r="C37" s="40"/>
+      <x:c r="D37" s="40"/>
+      <x:c r="E37" s="40"/>
+      <x:c r="F37" s="40"/>
+      <x:c r="G37" s="40"/>
+      <x:c r="H37" s="40"/>
+      <x:c r="I37" s="40"/>
+      <x:c r="J37" s="40"/>
+      <x:c r="K37" s="40"/>
+      <x:c r="L37" s="40"/>
+      <x:c r="M37" s="40"/>
+      <x:c r="N37" s="40"/>
+      <x:c r="O37" s="40"/>
+      <x:c r="P37" s="40"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="45" t="str">
+        <x:v>LINKED OUTPUTS | MIXED-INCOME CASE</x:v>
+      </x:c>
+      <x:c r="B38" s="45"/>
+      <x:c r="C38" s="45"/>
+      <x:c r="D38" s="45"/>
+      <x:c r="E38" s="45"/>
+      <x:c r="F38" s="45"/>
+      <x:c r="G38" s="45"/>
+      <x:c r="H38" s="45"/>
+      <x:c r="I38" s="45"/>
+      <x:c r="J38" s="45"/>
+      <x:c r="K38" s="45"/>
+      <x:c r="L38" s="45"/>
+      <x:c r="M38" s="45"/>
+      <x:c r="N38" s="45"/>
+      <x:c r="O38" s="45"/>
+      <x:c r="P38" s="45"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="40" t="str">
+        <x:v>Restricted rent potential / year</x:v>
+      </x:c>
+      <x:c r="B39" s="70" t="n">
+        <x:f>I34</x:f>
+        <x:v>456192</x:v>
+      </x:c>
+      <x:c r="C39" s="40"/>
+      <x:c r="D39" s="47" t="str">
+        <x:v>VOUCHER BASIS</x:v>
+      </x:c>
+      <x:c r="E39" s="47" t="str">
+        <x:v>INDICATED VALUE</x:v>
+      </x:c>
+      <x:c r="F39" s="47" t="str">
+        <x:v>GAP TO COST</x:v>
+      </x:c>
+      <x:c r="G39" s="40"/>
+      <x:c r="H39" s="40"/>
+      <x:c r="I39" s="40"/>
+      <x:c r="J39" s="40"/>
+      <x:c r="K39" s="40"/>
+      <x:c r="L39" s="40"/>
+      <x:c r="M39" s="40"/>
+      <x:c r="N39" s="40"/>
+      <x:c r="O39" s="40"/>
+      <x:c r="P39" s="40"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="40" t="str">
+        <x:v>Voucher rent potential / year</x:v>
+      </x:c>
+      <x:c r="B40" s="70" t="n">
+        <x:f>O34</x:f>
+        <x:v>168456</x:v>
+      </x:c>
+      <x:c r="C40" s="40"/>
+      <x:c r="D40" s="40" t="str">
+        <x:v>BHA 02135 benchmark</x:v>
+      </x:c>
+      <x:c r="E40" s="70" t="n">
+        <x:f>'Pro Forma'!C35+(SUMPRODUCT($D$31:$D$33,$L$31:$L$33)*12-$O$34)*(1-Inputs!$B$17)*(1-Inputs!$B$28)/(Inputs!$B$29+Inputs!$B$33)</x:f>
+        <x:v>66236934.22166558</x:v>
+      </x:c>
+      <x:c r="F40" s="70" t="n">
+        <x:f>MAX(0,'Pro Forma'!C17-E40)</x:f>
+        <x:v>13045418.71951089</x:v>
+      </x:c>
+      <x:c r="G40" s="40"/>
+      <x:c r="H40" s="40"/>
+      <x:c r="I40" s="40"/>
+      <x:c r="J40" s="40"/>
+      <x:c r="K40" s="40"/>
+      <x:c r="L40" s="40"/>
+      <x:c r="M40" s="40"/>
+      <x:c r="N40" s="40"/>
+      <x:c r="O40" s="40"/>
+      <x:c r="P40" s="40"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="40" t="str">
+        <x:v>Market rent potential / year</x:v>
+      </x:c>
+      <x:c r="B41" s="70" t="n">
+        <x:f>E34*Inputs!$B$14*12</x:f>
+        <x:v>5533500</x:v>
+      </x:c>
+      <x:c r="C41" s="40"/>
+      <x:c r="D41" s="40" t="str">
+        <x:v>Market-rent proxy</x:v>
+      </x:c>
+      <x:c r="E41" s="70" t="n">
+        <x:f>'Pro Forma'!C35+($D$34*Inputs!$B$14*12-$O$34)*(1-Inputs!$B$17)*(1-Inputs!$B$28)/(Inputs!$B$29+Inputs!$B$33)</x:f>
+        <x:v>67151579.09799068</x:v>
+      </x:c>
+      <x:c r="F41" s="70" t="n">
+        <x:f>MAX(0,'Pro Forma'!C17-E41)</x:f>
+        <x:v>12130773.843185797</x:v>
+      </x:c>
+      <x:c r="G41" s="40"/>
+      <x:c r="H41" s="40"/>
+      <x:c r="I41" s="40"/>
+      <x:c r="J41" s="40"/>
+      <x:c r="K41" s="40"/>
+      <x:c r="L41" s="40"/>
+      <x:c r="M41" s="40"/>
+      <x:c r="N41" s="40"/>
+      <x:c r="O41" s="40"/>
+      <x:c r="P41" s="40"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="47" t="str">
+        <x:v>Total residential GPR / year</x:v>
+      </x:c>
+      <x:c r="B42" s="75" t="n">
+        <x:f>SUM(B39:B41)</x:f>
+        <x:v>6158148</x:v>
+      </x:c>
+      <x:c r="C42" s="40"/>
+      <x:c r="D42" s="72" t="str">
+        <x:v>Gap range, low / high</x:v>
+      </x:c>
+      <x:c r="E42" s="73" t="n">
+        <x:f>MIN(F40:F41)</x:f>
+        <x:v>12130773.843185797</x:v>
+      </x:c>
+      <x:c r="F42" s="73" t="n">
+        <x:f>MAX(F40:F41)</x:f>
+        <x:v>13045418.71951089</x:v>
+      </x:c>
+      <x:c r="G42" s="40"/>
+      <x:c r="H42" s="40"/>
+      <x:c r="I42" s="40"/>
+      <x:c r="J42" s="40"/>
+      <x:c r="K42" s="40"/>
+      <x:c r="L42" s="40"/>
+      <x:c r="M42" s="40"/>
+      <x:c r="N42" s="40"/>
+      <x:c r="O42" s="40"/>
+      <x:c r="P42" s="40"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="52" t="str">
+        <x:v>Annual model NOI after tax</x:v>
+      </x:c>
+      <x:c r="B43" s="71" t="n">
+        <x:f>'Lease Economics'!C26</x:f>
+        <x:v>3444320.57952661</x:v>
+      </x:c>
+      <x:c r="C43" s="40"/>
+      <x:c r="D43" s="72" t="str">
+        <x:v>Incremental gap / designated home</x:v>
+      </x:c>
+      <x:c r="E43" s="73" t="n">
+        <x:f>'Pro Forma'!C40</x:f>
+        <x:v>318902.52437640127</x:v>
+      </x:c>
+      <x:c r="F43" s="73"/>
+      <x:c r="G43" s="40"/>
+      <x:c r="H43" s="40"/>
+      <x:c r="I43" s="40"/>
+      <x:c r="J43" s="40"/>
+      <x:c r="K43" s="40"/>
+      <x:c r="L43" s="40"/>
+      <x:c r="M43" s="40"/>
+      <x:c r="N43" s="40"/>
+      <x:c r="O43" s="40"/>
+      <x:c r="P43" s="40"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="52" t="str">
+        <x:v>Indicated stabilized value</x:v>
+      </x:c>
+      <x:c r="B44" s="71" t="n">
+        <x:f>'Pro Forma'!C35</x:f>
+        <x:v>66236934.22166558</x:v>
+      </x:c>
+      <x:c r="C44" s="40"/>
+      <x:c r="D44" s="40" t="str">
+        <x:v>Benchmarks only; approved voucher contracts and actual utility allowances are unknown.</x:v>
+      </x:c>
+      <x:c r="E44" s="40"/>
+      <x:c r="F44" s="40"/>
+      <x:c r="G44" s="40"/>
+      <x:c r="H44" s="40"/>
+      <x:c r="I44" s="40"/>
+      <x:c r="J44" s="40"/>
+      <x:c r="K44" s="40"/>
+      <x:c r="L44" s="40"/>
+      <x:c r="M44" s="40"/>
+      <x:c r="N44" s="40"/>
+      <x:c r="O44" s="40"/>
+      <x:c r="P44" s="40"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="52" t="str">
+        <x:v>Development funding gap</x:v>
+      </x:c>
+      <x:c r="B45" s="71" t="n">
+        <x:f>'Pro Forma'!C39</x:f>
+        <x:v>13045418.71951089</x:v>
+      </x:c>
+      <x:c r="C45" s="40"/>
+      <x:c r="D45" s="40" t="str">
+        <x:v>The incremental gap is NOT a subsidy amount or project funding request.</x:v>
+      </x:c>
+      <x:c r="E45" s="40"/>
+      <x:c r="F45" s="40"/>
+      <x:c r="G45" s="40"/>
+      <x:c r="H45" s="40"/>
+      <x:c r="I45" s="40"/>
+      <x:c r="J45" s="40"/>
+      <x:c r="K45" s="40"/>
+      <x:c r="L45" s="40"/>
+      <x:c r="M45" s="40"/>
+      <x:c r="N45" s="40"/>
+      <x:c r="O45" s="40"/>
+      <x:c r="P45" s="40"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="52" t="str">
+        <x:v>Yield on cost</x:v>
+      </x:c>
+      <x:c r="B46" s="54" t="n">
+        <x:f>'Pro Forma'!C36</x:f>
+        <x:v>0.043443722994474236</x:v>
+      </x:c>
+      <x:c r="C46" s="40"/>
+      <x:c r="D46" s="40"/>
+      <x:c r="E46" s="40"/>
+      <x:c r="F46" s="40"/>
+      <x:c r="G46" s="40"/>
+      <x:c r="H46" s="40"/>
+      <x:c r="I46" s="40"/>
+      <x:c r="J46" s="40"/>
+      <x:c r="K46" s="40"/>
+      <x:c r="L46" s="40"/>
+      <x:c r="M46" s="40"/>
+      <x:c r="N46" s="40"/>
+      <x:c r="O46" s="40"/>
+      <x:c r="P46" s="40"/>
+    </x:row>
+    <x:row r="47" ht="25" customHeight="1">
+      <x:c r="A47" s="45" t="str">
+        <x:v>SOURCES AND BOUNDARIES</x:v>
+      </x:c>
+      <x:c r="B47" s="45"/>
+      <x:c r="C47" s="45"/>
+      <x:c r="D47" s="45"/>
+      <x:c r="E47" s="45"/>
+      <x:c r="F47" s="45"/>
+      <x:c r="G47" s="45"/>
+      <x:c r="H47" s="45"/>
+      <x:c r="I47" s="45"/>
+      <x:c r="J47" s="45"/>
+      <x:c r="K47" s="45"/>
+      <x:c r="L47" s="45"/>
+      <x:c r="M47" s="45"/>
+      <x:c r="N47" s="45"/>
+      <x:c r="O47" s="45"/>
+      <x:c r="P47" s="45"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="76" t="str">
+        <x:v>City 2025 maximum affordable rents, 60% AMI; standard size, Studio / 1BR / 2BR: $1,266 / $1,484 / $1,680.</x:v>
+      </x:c>
+      <x:c r="B48" s="76"/>
+      <x:c r="C48" s="76"/>
+      <x:c r="D48" s="76"/>
+      <x:c r="E48" s="76"/>
+      <x:c r="F48" s="76"/>
+      <x:c r="G48" s="76"/>
+      <x:c r="H48" s="76"/>
+      <x:c r="I48" s="76"/>
+      <x:c r="J48" s="76"/>
+      <x:c r="K48" s="76"/>
+      <x:c r="L48" s="76"/>
+      <x:c r="M48" s="76"/>
+      <x:c r="N48" s="76"/>
+      <x:c r="O48" s="76"/>
+      <x:c r="P48" s="76"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="76" t="str">
+        <x:v>https://www.boston.gov/sites/default/files/file/2025/08/Income%20%26%20Rent%20Limits_August%204%2C%202025%20-%20AMI_%20Rent_%20Sales%20-%20All%20IDP.pdf</x:v>
+      </x:c>
+      <x:c r="B49" s="76"/>
+      <x:c r="C49" s="76"/>
+      <x:c r="D49" s="76"/>
+      <x:c r="E49" s="76"/>
+      <x:c r="F49" s="76"/>
+      <x:c r="G49" s="76"/>
+      <x:c r="H49" s="76"/>
+      <x:c r="I49" s="76"/>
+      <x:c r="J49" s="76"/>
+      <x:c r="K49" s="76"/>
+      <x:c r="L49" s="76"/>
+      <x:c r="M49" s="76"/>
+      <x:c r="N49" s="76"/>
+      <x:c r="O49" s="76"/>
+      <x:c r="P49" s="76"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="76" t="str">
+        <x:v>BHA payment standards effective Jan 1 2026, ZIP 02135, Studio / 1BR / 2BR: $2,627 / $2,757 / $3,270.</x:v>
+      </x:c>
+      <x:c r="B50" s="76"/>
+      <x:c r="C50" s="76"/>
+      <x:c r="D50" s="76"/>
+      <x:c r="E50" s="76"/>
+      <x:c r="F50" s="76"/>
+      <x:c r="G50" s="76"/>
+      <x:c r="H50" s="76"/>
+      <x:c r="I50" s="76"/>
+      <x:c r="J50" s="76"/>
+      <x:c r="K50" s="76"/>
+      <x:c r="L50" s="76"/>
+      <x:c r="M50" s="76"/>
+      <x:c r="N50" s="76"/>
+      <x:c r="O50" s="76"/>
+      <x:c r="P50" s="76"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="76" t="str">
+        <x:v>https://www.bostonhousing.org/BHA/media/Documents/Leased%20Housing/SAFMRs/2026-Payment-Standards-All-BR.pdf</x:v>
+      </x:c>
+      <x:c r="B51" s="76"/>
+      <x:c r="C51" s="76"/>
+      <x:c r="D51" s="76"/>
+      <x:c r="E51" s="76"/>
+      <x:c r="F51" s="76"/>
+      <x:c r="G51" s="76"/>
+      <x:c r="H51" s="76"/>
+      <x:c r="I51" s="76"/>
+      <x:c r="J51" s="76"/>
+      <x:c r="K51" s="76"/>
+      <x:c r="L51" s="76"/>
+      <x:c r="M51" s="76"/>
+      <x:c r="N51" s="76"/>
+      <x:c r="O51" s="76"/>
+      <x:c r="P51" s="76"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="76" t="str">
+        <x:v>Policy: https://www.boston.gov/departments/housing/inclusionary-zoning | BHA notes standards are NOT suggested contract rents.</x:v>
+      </x:c>
+      <x:c r="B52" s="76"/>
+      <x:c r="C52" s="76"/>
+      <x:c r="D52" s="76"/>
+      <x:c r="E52" s="76"/>
+      <x:c r="F52" s="76"/>
+      <x:c r="G52" s="76"/>
+      <x:c r="H52" s="76"/>
+      <x:c r="I52" s="76"/>
+      <x:c r="J52" s="76"/>
+      <x:c r="K52" s="76"/>
+      <x:c r="L52" s="76"/>
+      <x:c r="M52" s="76"/>
+      <x:c r="N52" s="76"/>
+      <x:c r="O52" s="76"/>
+      <x:c r="P52" s="76"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="76" t="str">
+        <x:v>Open items: actual Hew bedroom mix, 2026 IZ schedule, AMI distribution, utilities, contract rents, project-specific approval.</x:v>
+      </x:c>
+      <x:c r="B53" s="76"/>
+      <x:c r="C53" s="76"/>
+      <x:c r="D53" s="76"/>
+      <x:c r="E53" s="76"/>
+      <x:c r="F53" s="76"/>
+      <x:c r="G53" s="76"/>
+      <x:c r="H53" s="76"/>
+      <x:c r="I53" s="76"/>
+      <x:c r="J53" s="76"/>
+      <x:c r="K53" s="76"/>
+      <x:c r="L53" s="76"/>
+      <x:c r="M53" s="76"/>
+      <x:c r="N53" s="76"/>
+      <x:c r="O53" s="76"/>
+      <x:c r="P53" s="76"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="whole" operator="between" sqref="B21">
+      <x:formula1>1</x:formula1>
+      <x:formula2>2</x:formula2>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1285,19 +2898,20 @@
         <x:v>Affordable rent / home / month</x:v>
       </x:c>
       <x:c r="B15" s="19" t="n">
-        <x:v>1440</x:v>
+        <x:f>'Affordable Housing'!H34</x:f>
+        <x:v>1462.1538461538462</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
         <x:v>USD / month</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>Original 2025 rent proxy</x:v>
+        <x:v>City of Boston 2025 IDP, 60% AMI; modeled bedroom-weighted proxy</x:v>
       </x:c>
       <x:c r="E15" s="1" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>BENCHMARK / ASSUMED UNIT MIX</x:v>
       </x:c>
       <x:c r="F15" s="1" t="str">
-        <x:v>Must update to 2026 AMI, utilities and actual bedroom distribution</x:v>
+        <x:v>2025 City limits only; 2026 IDP limit, actual AMI mix and utility adjustments unverified. See Affordable Housing.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
@@ -1357,7 +2971,7 @@
         <x:v>Official framework</x:v>
       </x:c>
       <x:c r="F18" s="1" t="str">
-        <x:v>https://www.bostonplans.org/projects/standards/inclusionary-development-policy</x:v>
+        <x:v>150-home Option B illustrative new development; separate from Hew 2024 actual policy history.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
@@ -1377,7 +2991,7 @@
         <x:v>Official framework</x:v>
       </x:c>
       <x:c r="F19" s="1" t="str">
-        <x:v>https://www.bostonplans.org/projects/standards/inclusionary-development-policy</x:v>
+        <x:v>Unit shares require discrete rounding; this workbook uses illustrative 26 restricted + 5 voucher.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
@@ -1487,7 +3101,7 @@
         <x:v>UNVERIFIED</x:v>
       </x:c>
       <x:c r="F25" s="1" t="str">
-        <x:v>Assumed participation rate; the complete new-lease channel mix is unavailable.</x:v>
+        <x:v>Scenario assumption only; actual building-level broker share remains unknown.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
@@ -2069,7 +3683,7 @@
       </x:c>
       <x:c r="C6" s="3" t="n">
         <x:f>C5-C7-C8</x:f>
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D6" s="4"/>
     </x:row>
@@ -2082,11 +3696,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="3" t="n">
-        <x:f>ROUND(C5*Inputs!$B$18,0)</x:f>
+        <x:f>'Affordable Housing'!C34</x:f>
         <x:v>26</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Rounded from 17% of project</x:v>
+        <x:v>26 restricted homes in illustrative 150-home mix; 17% rounds up from 25.5.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
@@ -2098,11 +3712,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="3" t="n">
-        <x:f>ROUND(C5*(Inputs!$B$18+Inputs!$B$19),0)-C7</x:f>
-        <x:v>4</x:v>
+        <x:f>'Affordable Housing'!D34</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D8" s="4" t="str">
-        <x:v>3% voucher units use an UNVERIFIED market-rent proxy, not official SAFMR</x:v>
+        <x:v>5 voucher homes; 3% rounds up from 4.5 under modeled method; NOT a City ruling.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
@@ -2114,10 +3728,12 @@
         <x:v>6975000</x:v>
       </x:c>
       <x:c r="C9" s="3" t="n">
-        <x:f>(C6+C8)*Inputs!$B$14*12</x:f>
-        <x:v>5766000</x:v>
-      </x:c>
-      <x:c r="D9" s="4"/>
+        <x:f>C6*Inputs!$B$14*12+'Affordable Housing'!O34</x:f>
+        <x:v>5701956</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Market housing + separate voucher schedule; selected BHA/market proxy on Affordable Housing tab.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="1" t="str">
@@ -2128,10 +3744,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="3" t="n">
-        <x:f>C7*Inputs!$B$15*12</x:f>
-        <x:v>449280</x:v>
-      </x:c>
-      <x:c r="D10" s="4"/>
+        <x:f>'Affordable Housing'!I34</x:f>
+        <x:v>456192</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Weighted 2025 IDP 60% AMI limits for assumed Studio/1BR/2BR mix; utilities may reduce rent.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="9" t="str">
@@ -2143,7 +3761,7 @@
       </x:c>
       <x:c r="C11" s="10" t="n">
         <x:f>SUM(C9:C10)</x:f>
-        <x:v>6215280</x:v>
+        <x:v>6158148</x:v>
       </x:c>
       <x:c r="D11" s="12"/>
     </x:row>
@@ -2157,7 +3775,7 @@
       </x:c>
       <x:c r="C12" s="3" t="n">
         <x:f>-C11*Inputs!$B$17</x:f>
-        <x:v>-310764</x:v>
+        <x:v>-307907.4</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
         <x:v>Vacancy scenario is not public-listing availability</x:v>
@@ -2173,7 +3791,7 @@
       </x:c>
       <x:c r="C13" s="24" t="n">
         <x:f>C6*(1-Inputs!$B$17)</x:f>
-        <x:v>114</x:v>
+        <x:v>113.05</x:v>
       </x:c>
       <x:c r="D13" s="4"/>
     </x:row>
@@ -2187,7 +3805,7 @@
       </x:c>
       <x:c r="C14" s="24" t="n">
         <x:f>C13*Inputs!$B$21</x:f>
-        <x:v>51.300000000000004</x:v>
+        <x:v>50.8725</x:v>
       </x:c>
       <x:c r="D14" s="4"/>
     </x:row>
@@ -2201,7 +3819,7 @@
       </x:c>
       <x:c r="C15" s="24" t="n">
         <x:f>C13*(1-Inputs!$B$21)</x:f>
-        <x:v>62.7</x:v>
+        <x:v>62.1775</x:v>
       </x:c>
       <x:c r="D15" s="4"/>
     </x:row>
@@ -2215,7 +3833,7 @@
       </x:c>
       <x:c r="C16" s="3" t="n">
         <x:f>-C14*Inputs!$B$14*Inputs!$B$22</x:f>
-        <x:v>-397575.00000000006</x:v>
+        <x:v>-394261.875</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
         <x:v>Only new unrestricted market leases receive modeled free rent</x:v>
@@ -2231,7 +3849,7 @@
       </x:c>
       <x:c r="C17" s="3" t="n">
         <x:f>-C15*Inputs!$B$23*Inputs!$B$14*Inputs!$B$24</x:f>
-        <x:v>-60740.625</x:v>
+        <x:v>-60234.453125</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
         <x:v>Only selected renewals; historic one-month offer from May 2026</x:v>
@@ -2247,7 +3865,7 @@
       </x:c>
       <x:c r="C18" s="10" t="n">
         <x:f>SUM(C11:C12)+SUM(C16:C17)</x:f>
-        <x:v>5446200.375</x:v>
+        <x:v>5395744.271875</x:v>
       </x:c>
       <x:c r="D18" s="12"/>
     </x:row>
@@ -2277,7 +3895,7 @@
       </x:c>
       <x:c r="C20" s="10" t="n">
         <x:f>C18+C19</x:f>
-        <x:v>5446200.375</x:v>
+        <x:v>5395744.271875</x:v>
       </x:c>
       <x:c r="D20" s="12"/>
     </x:row>
@@ -2291,7 +3909,7 @@
       </x:c>
       <x:c r="C21" s="3" t="n">
         <x:f>-C20*Inputs!$B$28</x:f>
-        <x:v>-163386.01124999998</x:v>
+        <x:v>-161872.32815624998</x:v>
       </x:c>
       <x:c r="D21" s="4"/>
     </x:row>
@@ -2319,7 +3937,7 @@
       </x:c>
       <x:c r="C23" s="10" t="n">
         <x:f>SUM(C20:C22)</x:f>
-        <x:v>4322814.36375</x:v>
+        <x:v>4273871.94371875</x:v>
       </x:c>
       <x:c r="D23" s="12"/>
     </x:row>
@@ -2333,7 +3951,7 @@
       </x:c>
       <x:c r="C24" s="20" t="n">
         <x:f>IF(Inputs!$B$29+Inputs!$B$33&gt;0,C23/(Inputs!$B$29+Inputs!$B$33),"n.a.")</x:f>
-        <x:v>66995449.19332341</x:v>
+        <x:v>66236934.22166558</x:v>
       </x:c>
       <x:c r="D24" s="4" t="str">
         <x:v>NOI before tax / (capitalization rate + approximate property tax rate)</x:v>
@@ -2349,7 +3967,7 @@
       </x:c>
       <x:c r="C25" s="20" t="n">
         <x:f>-C24*Inputs!$B$33</x:f>
-        <x:v>-839051.0056971824</x:v>
+        <x:v>-829551.3641921398</x:v>
       </x:c>
       <x:c r="D25" s="4"/>
     </x:row>
@@ -2363,7 +3981,7 @@
       </x:c>
       <x:c r="C26" s="26" t="n">
         <x:f>C23+C25</x:f>
-        <x:v>3483763.358052817</x:v>
+        <x:v>3444320.57952661</x:v>
       </x:c>
       <x:c r="D26" s="12"/>
     </x:row>
@@ -2377,7 +3995,7 @@
       </x:c>
       <x:c r="C27" s="20" t="n">
         <x:f>IF(Inputs!$B$29&gt;0,C26/Inputs!$B$29,"n.a.")</x:f>
-        <x:v>66995449.19332341</x:v>
+        <x:v>66236934.22166558</x:v>
       </x:c>
       <x:c r="D27" s="4"/>
     </x:row>
@@ -2405,7 +4023,7 @@
       </x:c>
       <x:c r="C29" s="20" t="n">
         <x:f>-C14*Inputs!$B$14*Inputs!$B$25*Inputs!$B$26</x:f>
-        <x:v>-99393.75000000001</x:v>
+        <x:v>-98565.46875</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
         <x:v>Broker-sourced new leases only; separated from NOI for clarity</x:v>
@@ -2421,7 +4039,7 @@
       </x:c>
       <x:c r="C30" s="26" t="n">
         <x:f>SUM(C26,C28:C29)</x:f>
-        <x:v>3339369.608052817</x:v>
+        <x:v>3300755.11077661</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
         <x:v>Illustrative annual cash, not audited owner distributions</x:v>
@@ -2465,7 +4083,7 @@
       </x:c>
       <x:c r="C33" s="3" t="n">
         <x:f>C6*Inputs!$B$14*12*(1-Inputs!$B$17)+C16+C17</x:f>
-        <x:v>4842684.375</x:v>
+        <x:v>4802328.671875</x:v>
       </x:c>
       <x:c r="D33" s="4"/>
     </x:row>
@@ -2578,10 +4196,10 @@
       </x:c>
       <x:c r="C8" s="3" t="n">
         <x:f>'Lease Economics'!C8</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D8" s="4" t="str">
-        <x:v>Voucher rent proxied at market rent; verify actual SAFMR</x:v>
+        <x:v>2026 BHA benchmark or market proxy via Affordable Housing; neither is actual contract rent.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
@@ -2594,7 +4212,7 @@
       </x:c>
       <x:c r="C9" s="3" t="n">
         <x:f>'Lease Economics'!C6</x:f>
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D9" s="4"/>
     </x:row>
@@ -2736,7 +4354,7 @@
       </x:c>
       <x:c r="C20" s="20" t="n">
         <x:f>'Lease Economics'!C11</x:f>
-        <x:v>6215280</x:v>
+        <x:v>6158148</x:v>
       </x:c>
       <x:c r="D20" s="4"/>
     </x:row>
@@ -2750,7 +4368,7 @@
       </x:c>
       <x:c r="C21" s="20" t="n">
         <x:f>'Lease Economics'!C12</x:f>
-        <x:v>-310764</x:v>
+        <x:v>-307907.4</x:v>
       </x:c>
       <x:c r="D21" s="4"/>
     </x:row>
@@ -2764,7 +4382,7 @@
       </x:c>
       <x:c r="C22" s="20" t="n">
         <x:f>'Lease Economics'!C16</x:f>
-        <x:v>-397575.00000000006</x:v>
+        <x:v>-394261.875</x:v>
       </x:c>
       <x:c r="D22" s="4"/>
     </x:row>
@@ -2778,7 +4396,7 @@
       </x:c>
       <x:c r="C23" s="20" t="n">
         <x:f>'Lease Economics'!C17</x:f>
-        <x:v>-60740.625</x:v>
+        <x:v>-60234.453125</x:v>
       </x:c>
       <x:c r="D23" s="4"/>
     </x:row>
@@ -2806,7 +4424,7 @@
       </x:c>
       <x:c r="C25" s="26" t="n">
         <x:f>SUM(C20:C24)</x:f>
-        <x:v>5446200.375</x:v>
+        <x:v>5395744.271875</x:v>
       </x:c>
       <x:c r="D25" s="12"/>
     </x:row>
@@ -2834,7 +4452,7 @@
       </x:c>
       <x:c r="C27" s="20" t="n">
         <x:f>'Lease Economics'!C21</x:f>
-        <x:v>-163386.01124999998</x:v>
+        <x:v>-161872.32815624998</x:v>
       </x:c>
       <x:c r="D27" s="4"/>
     </x:row>
@@ -2848,7 +4466,7 @@
       </x:c>
       <x:c r="C28" s="20" t="n">
         <x:f>'Lease Economics'!C25</x:f>
-        <x:v>-839051.0056971824</x:v>
+        <x:v>-829551.3641921398</x:v>
       </x:c>
       <x:c r="D28" s="4"/>
     </x:row>
@@ -2862,7 +4480,7 @@
       </x:c>
       <x:c r="C29" s="26" t="n">
         <x:f>SUM(C25:C28)</x:f>
-        <x:v>3483763.358052817</x:v>
+        <x:v>3444320.57952661</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
         <x:v>Tax expense reconciles to loaded-cap valuation</x:v>
@@ -2892,7 +4510,7 @@
       </x:c>
       <x:c r="C31" s="20" t="n">
         <x:f>'Lease Economics'!C29</x:f>
-        <x:v>-99393.75000000001</x:v>
+        <x:v>-98565.46875</x:v>
       </x:c>
       <x:c r="D31" s="4"/>
     </x:row>
@@ -2906,7 +4524,7 @@
       </x:c>
       <x:c r="C32" s="26" t="n">
         <x:f>SUM(C29:C31)</x:f>
-        <x:v>3339369.608052817</x:v>
+        <x:v>3300755.11077661</x:v>
       </x:c>
       <x:c r="D32" s="12"/>
     </x:row>
@@ -2942,7 +4560,7 @@
       </x:c>
       <x:c r="C35" s="26" t="n">
         <x:f>'Lease Economics'!C24</x:f>
-        <x:v>66995449.19332341</x:v>
+        <x:v>66236934.22166558</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
         <x:v>Illustrative model indication, not an appraisal or Hew value</x:v>
@@ -2958,7 +4576,7 @@
       </x:c>
       <x:c r="C36" s="27" t="n">
         <x:f>C29/C17</x:f>
-        <x:v>0.04394122057196757</x:v>
+        <x:v>0.043443722994474236</x:v>
       </x:c>
       <x:c r="D36" s="4"/>
     </x:row>
@@ -2972,7 +4590,7 @@
       </x:c>
       <x:c r="C37" s="27" t="n">
         <x:f>C36-C34</x:f>
-        <x:v>-0.008058779428032431</x:v>
+        <x:v>-0.008556277005525761</x:v>
       </x:c>
       <x:c r="D37" s="4"/>
     </x:row>
@@ -2986,7 +4604,7 @@
       </x:c>
       <x:c r="C38" s="26" t="n">
         <x:f>C35-C17</x:f>
-        <x:v>-12286903.747853063</x:v>
+        <x:v>-13045418.71951089</x:v>
       </x:c>
       <x:c r="D38" s="12"/>
     </x:row>
@@ -3000,24 +4618,24 @@
       </x:c>
       <x:c r="C39" s="26" t="n">
         <x:f>MAX(0,-C38)</x:f>
-        <x:v>12286903.747853063</x:v>
+        <x:v>13045418.71951089</x:v>
       </x:c>
       <x:c r="D39" s="12"/>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
       <x:c r="A40" s="1" t="str">
-        <x:v>Funding gap / restricted home</x:v>
+        <x:v>Incremental value-to-cost gap per designated home</x:v>
       </x:c>
       <x:c r="B40" s="20" t="n">
         <x:f>0</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
-        <x:f>IF(C7&gt;0,C39/C7,"n.a.")</x:f>
-        <x:v>472573.22107127163</x:v>
+        <x:f>IF(SUM(C7:C8)&gt;0,(C39-B39)/SUM(C7:C8),0)</x:f>
+        <x:v>318902.52437640127</x:v>
       </x:c>
       <x:c r="D40" s="4" t="str">
-        <x:v>Not an IDP-approved subsidy amount</x:v>
+        <x:v>(Mixed-income gap - market-rate gap) / 31 designated homes. NOT subsidy per affordable unit.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
@@ -3457,7 +5075,7 @@
         <x:v>3913391.4488213686</x:v>
       </x:c>
       <x:c r="D33" s="3" t="str">
-        <x:v>Scenario assumption; the complete new-lease channel mix is unavailable.</x:v>
+        <x:v>Not a measured broker share; deals from one brokerage do not supply total channel mix</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="20" customHeight="1">
@@ -3473,7 +5091,7 @@
         <x:v>3851270.3550713686</x:v>
       </x:c>
       <x:c r="D34" s="3" t="str">
-        <x:v>Scenario assumption; the complete new-lease channel mix is unavailable.</x:v>
+        <x:v>Not a measured broker share; deals from one brokerage do not supply total channel mix</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="20" customHeight="1">
@@ -3489,7 +5107,7 @@
         <x:v>3789149.2613213686</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
-        <x:v>Scenario assumption; the complete new-lease channel mix is unavailable.</x:v>
+        <x:v>Not a measured broker share; deals from one brokerage do not supply total channel mix</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
@@ -3505,7 +5123,7 @@
         <x:v>3727028.1675713686</x:v>
       </x:c>
       <x:c r="D36" s="3" t="str">
-        <x:v>Scenario assumption; the complete new-lease channel mix is unavailable.</x:v>
+        <x:v>Not a measured broker share; deals from one brokerage do not supply total channel mix</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
@@ -3521,7 +5139,7 @@
         <x:v>3664907.0738213686</x:v>
       </x:c>
       <x:c r="D37" s="3" t="str">
-        <x:v>Scenario assumption; the complete new-lease channel mix is unavailable.</x:v>
+        <x:v>Not a measured broker share; deals from one brokerage do not supply total channel mix</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
@@ -3828,19 +5446,33 @@
       <x:c r="H16" s="1"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="1"/>
-      <x:c r="B17" s="1"/>
-      <x:c r="C17" s="1"/>
-      <x:c r="D17" s="1"/>
-      <x:c r="E17" s="1"/>
-      <x:c r="F17" s="1"/>
-      <x:c r="G17" s="1"/>
-      <x:c r="H17" s="1"/>
+      <x:c r="A17" s="1" t="str">
+        <x:v>Full-property broker-sourced lease count</x:v>
+      </x:c>
+      <x:c r="B17" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="str">
+        <x:v>not verified</x:v>
+      </x:c>
+      <x:c r="D17" s="1" t="str"/>
+      <x:c r="E17" s="1" t="str"/>
+      <x:c r="F17" s="1" t="str"/>
+      <x:c r="G17" s="1" t="str"/>
+      <x:c r="H17" s="1" t="str">
+        <x:v>No authoritative full-property lease ledger or broker-channel breakdown; company-level production not published.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="1"/>
-      <x:c r="B18" s="27"/>
-      <x:c r="C18" s="1"/>
+      <x:c r="A18" s="1" t="str">
+        <x:v>Property-wide lease turnover and broker share</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Not verified from public data</x:v>
+      </x:c>
       <x:c r="D18" s="1"/>
       <x:c r="E18" s="1"/>
       <x:c r="F18" s="1"/>
@@ -4916,24 +6548,20 @@
       <x:c r="D29" s="3"/>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
-      <x:c r="A30" s="1" t="str">
-        <x:v>Building-wide turnover and broker-sourced share are unavailable.</x:v>
-      </x:c>
+      <x:c r="A30" s="1"/>
       <x:c r="B30" s="3"/>
       <x:c r="C30" s="3"/>
       <x:c r="D30" s="3"/>
     </x:row>
     <x:row r="31" ht="20" customHeight="1">
-      <x:c r="A31" s="1" t="str">
-        <x:v>Public edition excludes confidential transaction records.</x:v>
-      </x:c>
+      <x:c r="A31" s="1"/>
       <x:c r="B31" s="3"/>
       <x:c r="C31" s="3"/>
       <x:c r="D31" s="3"/>
     </x:row>
     <x:row r="32" ht="20" customHeight="1">
       <x:c r="A32" s="1" t="str">
-        <x:v>Voucher-rent market proxy requires project-specific SAFMR verification and cannot be called policy-compliant.</x:v>
+        <x:v>2026 BHA ZIP 02135 payment standards are public but are NOT approved owner rents; voucher mode is illustrative.</x:v>
       </x:c>
       <x:c r="B32" s="3"/>
       <x:c r="C32" s="3"/>
@@ -4941,7 +6569,7 @@
     </x:row>
     <x:row r="33" ht="20" customHeight="1">
       <x:c r="A33" s="1" t="str">
-        <x:v>The 17% restricted + 3% voucher policy is one large-project option, not a legal conclusion about Hew or other sites.</x:v>
+        <x:v>The 17% + 3% Option B is a hypothetical post-2024 site case; rounding, AMI distribution and compliance need official review.</x:v>
       </x:c>
       <x:c r="B33" s="3"/>
       <x:c r="C33" s="3"/>
@@ -4970,10 +6598,217 @@
       <x:c r="D36" s="3"/>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
-      <x:c r="A37" s="1"/>
-      <x:c r="B37" s="3"/>
-      <x:c r="C37" s="3"/>
-      <x:c r="D37" s="3"/>
+      <x:c r="A37" s="79" t="str">
+        <x:v>MIXED-INCOME HOUSING / VOUCHER AUDIT</x:v>
+      </x:c>
+      <x:c r="B37" s="80"/>
+      <x:c r="C37" s="80"/>
+      <x:c r="D37" s="80"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="40" t="str">
+        <x:v>Total home count</x:v>
+      </x:c>
+      <x:c r="B38" s="81" t="n">
+        <x:f>'Affordable Housing'!B34-Inputs!$B$6</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C38" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D38" s="40" t="str">
+        <x:v>Selected bedroom inventory must equal total project units.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="40" t="str">
+        <x:v>Restricted unit count</x:v>
+      </x:c>
+      <x:c r="B39" s="81" t="n">
+        <x:f>'Affordable Housing'!C34-'Affordable Housing'!B11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C39" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="40" t="str">
+        <x:v>26 restricted homes; model uses independently rounded 17%.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="40" t="str">
+        <x:v>Voucher unit count</x:v>
+      </x:c>
+      <x:c r="B40" s="81" t="n">
+        <x:f>'Affordable Housing'!D34-'Affordable Housing'!B12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C40" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="40" t="str">
+        <x:v>5 vouchers; model uses independently rounded 3%.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="40" t="str">
+        <x:v>Bedroom-mix arithmetic</x:v>
+      </x:c>
+      <x:c r="B41" s="81" t="n">
+        <x:f>SUM('Affordable Housing'!P31:P33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C41" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="40" t="str">
+        <x:v>Each type: market + restricted + voucher must equal that bedroom count.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="40" t="str">
+        <x:v>Market unit count</x:v>
+      </x:c>
+      <x:c r="B42" s="81" t="n">
+        <x:f>'Lease Economics'!C6-'Affordable Housing'!E34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C42" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="40" t="str">
+        <x:v>119 market homes from the assumed mix.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="40" t="str">
+        <x:v>Restricted annual rent bridge</x:v>
+      </x:c>
+      <x:c r="B43" s="81" t="n">
+        <x:f>'Lease Economics'!C10-'Affordable Housing'!I34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C43" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D43" s="40" t="str">
+        <x:v>By-bedroom 2025 limits less entered utility allowance, if any.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="40" t="str">
+        <x:v>Voucher annual rent bridge</x:v>
+      </x:c>
+      <x:c r="B44" s="81" t="n">
+        <x:f>'Lease Economics'!C9-'Affordable Housing'!E34*Inputs!$B$14*12-'Affordable Housing'!O34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C44" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="40" t="str">
+        <x:v>Separate voucher rents, never untested default market rents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="40" t="str">
+        <x:v>Gross potential rent bridge</x:v>
+      </x:c>
+      <x:c r="B45" s="81" t="n">
+        <x:f>'Lease Economics'!C11-'Affordable Housing'!B42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C45" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="40" t="str">
+        <x:v>Market + restricted + voucher annual potential rents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="40" t="str">
+        <x:v>Voucher selector (1 or 2)</x:v>
+      </x:c>
+      <x:c r="B46" s="81" t="n">
+        <x:f>IF(OR('Affordable Housing'!B21=1,'Affordable Housing'!B21=2),0,1)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C46" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D46" s="40" t="str">
+        <x:v>0 = valid choice; 1 = invalid input.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="40" t="str">
+        <x:v>Restricted maximum threshold</x:v>
+      </x:c>
+      <x:c r="B47" s="81" t="n">
+        <x:f>SUM(MAX(0,'Affordable Housing'!H31-'Affordable Housing'!F31),MAX(0,'Affordable Housing'!H32-'Affordable Housing'!F32),MAX(0,'Affordable Housing'!H33-'Affordable Housing'!F33))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C47" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D47" s="40" t="str">
+        <x:v>Selected restricted net rents do not exceed entered table limits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="40" t="str">
+        <x:v>Restricted share minimum</x:v>
+      </x:c>
+      <x:c r="B48" s="81" t="n">
+        <x:f>MAX(0,ROUNDUP(Inputs!$B$6*Inputs!$B$18,0)-'Affordable Housing'!C34)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C48" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D48" s="40" t="str">
+        <x:v>0 means arithmetic round-up threshold met; NOT legal signoff.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="40" t="str">
+        <x:v>Voucher share minimum</x:v>
+      </x:c>
+      <x:c r="B49" s="81" t="n">
+        <x:f>MAX(0,ROUNDUP(Inputs!$B$6*Inputs!$B$19,0)-'Affordable Housing'!D34)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C49" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D49" s="40" t="str">
+        <x:v>0 means arithmetic round-up threshold met; NOT legal signoff.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="40" t="str">
+        <x:v>Incremental gap per designated unit</x:v>
+      </x:c>
+      <x:c r="B50" s="81" t="n">
+        <x:f>'Pro Forma'!C40-('Pro Forma'!C39-'Pro Forma'!B39)/SUM('Pro Forma'!C7:C8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C50" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D50" s="40" t="str">
+        <x:v>Subtract pre-existing market-rate gap; divide by 31, not just the 26 restricted homes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>STATUS: Arithmetic checks ≠ compliance. Verify 2026 published IDP rent limits, allowed AMI averages, compact units and utility allowances.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>BHA standards are gross and subject to reasonableness; default zero utility allowances do not represent verification.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>